<commit_message>
Add Honduras year-by-year table: productivity, fertiliser, rust, varieties, finance, lempira
New workbook and 6-slide deck with year-on-year changes 2005-2026:
yield per bearing hectare and per tree, FAOSTAT nitrogen and urea
imports, urea and coffee prices in lempiras (BCH daily rate), every
rust figure found, variety adoption, Bono Cafetalero and financing
programmes. FAOSTAT fertiliser use now runs to 2024 in the yield-driver
work (2022 imputed by FAO); stale 'stops in 2022' text corrected.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCSUFXh2mYdWNgg7VCeE1G
</commit_message>
<xml_diff>
--- a/research/honduras/excel/Honduras_yield_drivers_forecast.xlsx
+++ b/research/honduras/excel/Honduras_yield_drivers_forecast.xlsx
@@ -4867,7 +4867,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t xml:space="preserve">FAO nitrogen use is for all crops (coffee is not separated) and stops in 2022.</t>
+          <t xml:space="preserve">FAO nitrogen use is for all crops (coffee is not separated); it runs to 2024 and the 2022 value is imputed by FAO (flag I).</t>
         </is>
       </c>
     </row>
@@ -8369,10 +8369,10 @@
         <v>0.751</v>
       </c>
       <c r="D6" s="14">
-        <v>0.0004</v>
+        <v>0.0002</v>
       </c>
       <c r="E6" s="14">
-        <v>0.0056</v>
+        <v>0.0028</v>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
@@ -8397,10 +8397,10 @@
         <v>-0.521</v>
       </c>
       <c r="D7" s="14">
-        <v>0.0008</v>
+        <v>0.0004</v>
       </c>
       <c r="E7" s="14">
-        <v>0.010400000000000001</v>
+        <v>0.005200000000000001</v>
       </c>
       <c r="F7" s="15" t="inlineStr">
         <is>
@@ -8453,10 +8453,10 @@
         <v>0.344</v>
       </c>
       <c r="D9" s="14">
-        <v>0.0228</v>
+        <v>0.0234</v>
       </c>
       <c r="E9" s="14">
-        <v>0.2508</v>
+        <v>0.2574</v>
       </c>
       <c r="F9" s="16" t="inlineStr">
         <is>
@@ -8481,10 +8481,10 @@
         <v>0.33</v>
       </c>
       <c r="D10" s="14">
-        <v>0.03</v>
+        <v>0.0268</v>
       </c>
       <c r="E10" s="14">
-        <v>0.3</v>
+        <v>0.268</v>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
@@ -8509,10 +8509,10 @@
         <v>0.32</v>
       </c>
       <c r="D11" s="14">
-        <v>0.0358</v>
+        <v>0.0342</v>
       </c>
       <c r="E11" s="14">
-        <v>0.3222</v>
+        <v>0.3078</v>
       </c>
       <c r="F11" s="16" t="inlineStr">
         <is>
@@ -8533,7 +8533,7 @@
         <v>0.199</v>
       </c>
       <c r="D12" s="14">
-        <v>0.1998</v>
+        <v>0.201</v>
       </c>
       <c r="E12" s="14">
         <v>1</v>
@@ -8547,17 +8547,17 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rain Jun-Oct (fruit fill)</t>
+          <t xml:space="preserve">Rain Apr-May (flowering, fruit set)</t>
         </is>
       </c>
       <c r="B13">
         <v>44</v>
       </c>
       <c r="C13" s="13">
-        <v>0.101</v>
+        <v>-0.103</v>
       </c>
       <c r="D13" s="14">
-        <v>0.5065</v>
+        <v>0.5087</v>
       </c>
       <c r="E13" s="14">
         <v>1</v>
@@ -8568,38 +8568,38 @@
         </is>
       </c>
       <c r="G13" s="12">
+        <f>CORREL(Changes!D18:D61,Changes!K18:K61)</f>
+        <v>-0.10323980859597548</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Rain Jun-Oct (fruit fill)</t>
+        </is>
+      </c>
+      <c r="B14">
+        <v>44</v>
+      </c>
+      <c r="C14" s="13">
+        <v>0.101</v>
+      </c>
+      <c r="D14" s="14">
+        <v>0.5173</v>
+      </c>
+      <c r="E14" s="14">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no link</t>
+        </is>
+      </c>
+      <c r="G14" s="12">
         <f>CORREL(Changes!D18:D61,Changes!L18:L61)</f>
         <v>0.10143212443940035</v>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Rain Apr-May (flowering, fruit set)</t>
-        </is>
-      </c>
-      <c r="B14">
-        <v>44</v>
-      </c>
-      <c r="C14" s="13">
-        <v>-0.103</v>
-      </c>
-      <c r="D14" s="14">
-        <v>0.5089</v>
-      </c>
-      <c r="E14" s="14">
-        <v>1</v>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no link</t>
-        </is>
-      </c>
-      <c r="G14" s="12">
-        <f>CORREL(Changes!D18:D61,Changes!K18:K61)</f>
-        <v>-0.10323980859597548</v>
-      </c>
-    </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
@@ -8613,7 +8613,7 @@
         <v>-0.078</v>
       </c>
       <c r="D15" s="14">
-        <v>0.6279</v>
+        <v>0.6219</v>
       </c>
       <c r="E15" s="14">
         <v>1</v>
@@ -8637,7 +8637,7 @@
         <v>-0.07</v>
       </c>
       <c r="D16" s="14">
-        <v>0.6515</v>
+        <v>0.6441</v>
       </c>
       <c r="E16" s="14">
         <v>1</v>
@@ -8661,7 +8661,7 @@
         <v>-0.028</v>
       </c>
       <c r="D17" s="14">
-        <v>0.8594</v>
+        <v>0.8548</v>
       </c>
       <c r="E17" s="14">
         <v>1</v>
@@ -8685,7 +8685,7 @@
         <v>-0.01</v>
       </c>
       <c r="D18" s="14">
-        <v>0.951</v>
+        <v>0.9436</v>
       </c>
       <c r="E18" s="14">
         <v>1</v>
@@ -8713,7 +8713,7 @@
         <v>-0.009</v>
       </c>
       <c r="D19" s="14">
-        <v>0.955</v>
+        <v>0.9582</v>
       </c>
       <c r="E19" s="14">
         <v>1</v>
@@ -8785,14 +8785,14 @@
         <v>0.691</v>
       </c>
       <c r="D23" s="14">
-        <v>0.0044</v>
+        <v>0.0034</v>
       </c>
       <c r="E23" s="14">
-        <v>0.0616</v>
-      </c>
-      <c r="F23" s="16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">weak (p&lt;0.05 alone)</t>
+        <v>0.047599999999999996</v>
+      </c>
+      <c r="F23" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">robust</t>
         </is>
       </c>
       <c r="G23" s="12">
@@ -8813,10 +8813,10 @@
         <v>-0.411</v>
       </c>
       <c r="D24" s="14">
-        <v>0.0102</v>
+        <v>0.0098</v>
       </c>
       <c r="E24" s="14">
-        <v>0.1326</v>
+        <v>0.12739999999999999</v>
       </c>
       <c r="F24" s="16" t="inlineStr">
         <is>
@@ -8841,10 +8841,10 @@
         <v>0.335</v>
       </c>
       <c r="D25" s="14">
-        <v>0.0342</v>
+        <v>0.0398</v>
       </c>
       <c r="E25" s="14">
-        <v>0.4104</v>
+        <v>0.4776</v>
       </c>
       <c r="F25" s="16" t="inlineStr">
         <is>
@@ -8869,10 +8869,10 @@
         <v>0.308</v>
       </c>
       <c r="D26" s="14">
-        <v>0.0576</v>
+        <v>0.0532</v>
       </c>
       <c r="E26" s="14">
-        <v>0.6335999999999999</v>
+        <v>0.5851999999999999</v>
       </c>
       <c r="F26" s="16" t="inlineStr">
         <is>
@@ -8897,10 +8897,10 @@
         <v>0.305</v>
       </c>
       <c r="D27" s="14">
-        <v>0.0616</v>
+        <v>0.0586</v>
       </c>
       <c r="E27" s="14">
-        <v>0.6335999999999999</v>
+        <v>0.586</v>
       </c>
       <c r="F27" s="16" t="inlineStr">
         <is>
@@ -8925,7 +8925,7 @@
         <v>0.247</v>
       </c>
       <c r="D28" s="14">
-        <v>0.125</v>
+        <v>0.129</v>
       </c>
       <c r="E28" s="14">
         <v>1</v>
@@ -8953,7 +8953,7 @@
         <v>0.245</v>
       </c>
       <c r="D29" s="14">
-        <v>0.146</v>
+        <v>0.1312</v>
       </c>
       <c r="E29" s="14">
         <v>1</v>
@@ -8977,7 +8977,7 @@
         <v>-0.211</v>
       </c>
       <c r="D30" s="14">
-        <v>0.1964</v>
+        <v>0.1986</v>
       </c>
       <c r="E30" s="14">
         <v>1</v>
@@ -8995,17 +8995,17 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Max temperature Mar-May (NASA POWER)</t>
+          <t xml:space="preserve">Rain Apr-May (flowering, fruit set)</t>
         </is>
       </c>
       <c r="B31">
         <v>39</v>
       </c>
       <c r="C31" s="13">
-        <v>0.205</v>
+        <v>-0.204</v>
       </c>
       <c r="D31" s="14">
-        <v>0.2046</v>
+        <v>0.208</v>
       </c>
       <c r="E31" s="14">
         <v>1</v>
@@ -9015,21 +9015,25 @@
           <t xml:space="preserve">no link</t>
         </is>
       </c>
+      <c r="G31" s="12">
+        <f>CORREL(Changes!C18:C56,Changes!K18:K56)</f>
+        <v>-0.20418549530352773</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rain Apr-May (flowering, fruit set)</t>
+          <t xml:space="preserve">Max temperature Mar-May (NASA POWER)</t>
         </is>
       </c>
       <c r="B32">
         <v>39</v>
       </c>
       <c r="C32" s="13">
-        <v>-0.204</v>
+        <v>0.205</v>
       </c>
       <c r="D32" s="14">
-        <v>0.2108</v>
+        <v>0.2124</v>
       </c>
       <c r="E32" s="14">
         <v>1</v>
@@ -9039,10 +9043,6 @@
           <t xml:space="preserve">no link</t>
         </is>
       </c>
-      <c r="G32" s="12">
-        <f>CORREL(Changes!C18:C56,Changes!K18:K56)</f>
-        <v>-0.20418549530352773</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -9057,7 +9057,7 @@
         <v>-0.046</v>
       </c>
       <c r="D33" s="14">
-        <v>0.7822</v>
+        <v>0.7806</v>
       </c>
       <c r="E33" s="14">
         <v>1</v>
@@ -9081,7 +9081,7 @@
         <v>-0.03</v>
       </c>
       <c r="D34" s="14">
-        <v>0.845</v>
+        <v>0.8582</v>
       </c>
       <c r="E34" s="14">
         <v>1</v>
@@ -9109,7 +9109,7 @@
         <v>-0.02</v>
       </c>
       <c r="D35" s="14">
-        <v>0.905</v>
+        <v>0.8902</v>
       </c>
       <c r="E35" s="14">
         <v>1</v>
@@ -9133,7 +9133,7 @@
         <v>0.014</v>
       </c>
       <c r="D36" s="14">
-        <v>0.9348</v>
+        <v>0.9324</v>
       </c>
       <c r="E36" s="14">
         <v>1</v>
@@ -9201,10 +9201,10 @@
         <v>-0.573</v>
       </c>
       <c r="D40" s="14">
-        <v>0.0124</v>
+        <v>0.0108</v>
       </c>
       <c r="E40" s="14">
-        <v>0.1736</v>
+        <v>0.1512</v>
       </c>
       <c r="F40" s="16" t="inlineStr">
         <is>
@@ -9229,10 +9229,10 @@
         <v>0.557</v>
       </c>
       <c r="D41" s="14">
-        <v>0.0124</v>
+        <v>0.0136</v>
       </c>
       <c r="E41" s="14">
-        <v>0.1736</v>
+        <v>0.17679999999999998</v>
       </c>
       <c r="F41" s="16" t="inlineStr">
         <is>
@@ -9257,10 +9257,10 @@
         <v>0.437</v>
       </c>
       <c r="D42" s="14">
-        <v>0.0572</v>
+        <v>0.0578</v>
       </c>
       <c r="E42" s="14">
-        <v>0.6864</v>
+        <v>0.6936</v>
       </c>
       <c r="F42" s="16" t="inlineStr">
         <is>
@@ -9285,10 +9285,10 @@
         <v>0.407</v>
       </c>
       <c r="D43" s="14">
-        <v>0.0776</v>
+        <v>0.0736</v>
       </c>
       <c r="E43" s="14">
-        <v>0.8536</v>
+        <v>0.8096</v>
       </c>
       <c r="F43" s="16" t="inlineStr">
         <is>
@@ -9309,10 +9309,10 @@
         <v>0.406</v>
       </c>
       <c r="D44" s="14">
-        <v>0.0784</v>
+        <v>0.0752</v>
       </c>
       <c r="E44" s="14">
-        <v>0.8536</v>
+        <v>0.8096</v>
       </c>
       <c r="F44" s="16" t="inlineStr">
         <is>
@@ -9337,7 +9337,7 @@
         <v>-0.355</v>
       </c>
       <c r="D45" s="14">
-        <v>0.12</v>
+        <v>0.1248</v>
       </c>
       <c r="E45" s="14">
         <v>1</v>
@@ -9365,7 +9365,7 @@
         <v>0.334</v>
       </c>
       <c r="D46" s="14">
-        <v>0.1494</v>
+        <v>0.1468</v>
       </c>
       <c r="E46" s="14">
         <v>1</v>
@@ -9393,7 +9393,7 @@
         <v>0.306</v>
       </c>
       <c r="D47" s="14">
-        <v>0.1938</v>
+        <v>0.1902</v>
       </c>
       <c r="E47" s="14">
         <v>1</v>
@@ -9421,7 +9421,7 @@
         <v>0.265</v>
       </c>
       <c r="D48" s="14">
-        <v>0.2635</v>
+        <v>0.2613</v>
       </c>
       <c r="E48" s="14">
         <v>1</v>
@@ -9445,7 +9445,7 @@
         <v>-0.232</v>
       </c>
       <c r="D49" s="14">
-        <v>0.3301</v>
+        <v>0.3287</v>
       </c>
       <c r="E49" s="14">
         <v>1</v>
@@ -9469,7 +9469,7 @@
         <v>0.2</v>
       </c>
       <c r="D50" s="14">
-        <v>0.3883</v>
+        <v>0.3999</v>
       </c>
       <c r="E50" s="14">
         <v>1</v>
@@ -9497,7 +9497,7 @@
         <v>-0.166</v>
       </c>
       <c r="D51" s="14">
-        <v>0.4945</v>
+        <v>0.4805</v>
       </c>
       <c r="E51" s="14">
         <v>1</v>
@@ -9521,7 +9521,7 @@
         <v>-0.08</v>
       </c>
       <c r="D52" s="14">
-        <v>0.7353</v>
+        <v>0.7355</v>
       </c>
       <c r="E52" s="14">
         <v>1</v>
@@ -10954,131 +10954,143 @@
         <v>700.0333333333334</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2023/24</t>
+        </is>
+      </c>
+      <c r="B23" s="19">
+        <f>Data!K59</f>
+        <v>104427.0</v>
+      </c>
+      <c r="C23" s="11">
+        <f>Changes!I59</f>
+        <v>-0.004185545930430453</v>
+      </c>
+      <c r="D23" s="11">
+        <f>Changes!D59</f>
+        <v>-0.12107793155323604</v>
+      </c>
+      <c r="E23" s="12">
+        <f>Data!H59</f>
+        <v>4.540833333333333</v>
+      </c>
+      <c r="F23" s="19">
+        <f>Data!I59</f>
+        <v>358.0083333333334</v>
+      </c>
+    </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024/25</t>
+        </is>
+      </c>
+      <c r="B24" s="19">
+        <f>Data!K60</f>
+        <v>106830.0</v>
+      </c>
+      <c r="C24" s="11">
+        <f>Changes!I60</f>
+        <v>0.022750523256168362</v>
+      </c>
+      <c r="D24" s="11">
+        <f>Changes!D60</f>
+        <v>0.029270382300113237</v>
+      </c>
+      <c r="E24" s="12">
+        <f>Data!H60</f>
+        <v>5.620833333333333</v>
+      </c>
+      <c r="F24" s="19">
+        <f>Data!I60</f>
+        <v>338.28333333333336</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">r(N use change, production change)</t>
         </is>
       </c>
-      <c r="C24" s="12">
-        <f>CORREL(C5:C22,D5:D22)</f>
-        <v>0.7532522388489884</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="C26" s="12">
+        <f>CORREL(C5:C24,D5:D24)</f>
+        <v>0.7509896692236512</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
         <is>
           <t xml:space="preserve">Smallest r when any one year is left out (Python)</t>
         </is>
       </c>
-      <c r="C25" s="13">
-        <v>0.6900174039113661</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="C27" s="13">
+        <v>0.6924765127343235</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">What moves nitrogen use?</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">n</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">r</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">p (permutation)</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Verdict</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N use change vs output change, same crop year</t>
-        </is>
-      </c>
-      <c r="B28">
-        <v>18</v>
-      </c>
-      <c r="C28" s="13">
-        <v>0.7532522388489884</v>
-      </c>
-      <c r="D28" s="14">
-        <v>0.0003999200159968006</v>
-      </c>
-      <c r="E28" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">yes</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">N use change vs output change of the crop before (income)</t>
-        </is>
-      </c>
-      <c r="B29">
-        <v>18</v>
-      </c>
-      <c r="C29" s="13">
-        <v>-0.06605295740219877</v>
-      </c>
-      <c r="D29" s="14">
-        <v>0.7908418316336733</v>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">N use change vs world arabica price change, same calendar year</t>
+          <t xml:space="preserve">N use change vs output change, same crop year</t>
         </is>
       </c>
       <c r="B30">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C30" s="13">
-        <v>0.2803703387486554</v>
+        <v>0.7509896692236512</v>
       </c>
       <c r="D30" s="14">
-        <v>0.2465506898620276</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">no</t>
+        <v>0.0003999200159968006</v>
+      </c>
+      <c r="E30" s="15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">yes</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">N use change vs coffee/urea price ratio change</t>
+          <t xml:space="preserve">N use change vs output change of the crop before (income)</t>
         </is>
       </c>
       <c r="B31">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C31" s="13">
-        <v>0.22692652676931513</v>
+        <v>-0.06822334122020131</v>
       </c>
       <c r="D31" s="14">
-        <v>0.3693261347730454</v>
+        <v>0.769246150769846</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -11089,17 +11101,17 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">N use change vs urea price change</t>
+          <t xml:space="preserve">N use change vs world arabica price change, same calendar year</t>
         </is>
       </c>
       <c r="B32">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C32" s="13">
-        <v>-0.026533683105172953</v>
+        <v>0.2782930148974867</v>
       </c>
       <c r="D32" s="14">
-        <v>0.9154169166166767</v>
+        <v>0.2435512897420516</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -11110,42 +11122,84 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t xml:space="preserve">N use change vs coffee/urea price ratio change</t>
+        </is>
+      </c>
+      <c r="B33">
+        <v>20</v>
+      </c>
+      <c r="C33" s="13">
+        <v>0.1761195848332071</v>
+      </c>
+      <c r="D33" s="14">
+        <v>0.4513097380523895</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">N use change vs urea price change</t>
+        </is>
+      </c>
+      <c r="B34">
+        <v>20</v>
+      </c>
+      <c r="C34" s="13">
+        <v>0.016437183302314213</v>
+      </c>
+      <c r="D34" s="14">
+        <v>0.9498100379924015</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t xml:space="preserve">N use change vs IHCAFE export price change of the crop before</t>
         </is>
       </c>
-      <c r="B33">
+      <c r="B35">
         <v>17</v>
       </c>
-      <c r="C33" s="13">
+      <c r="C35" s="13">
         <v>0.46848608577687656</v>
       </c>
-      <c r="D33" s="14">
-        <v>0.05658868226354729</v>
-      </c>
-      <c r="E33" s="16" t="inlineStr">
+      <c r="D35" s="14">
+        <v>0.05538892221555689</v>
+      </c>
+      <c r="E35" s="16" t="inlineStr">
         <is>
           <t xml:space="preserve">hint</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Reading: nitrogen and output rise and fall together, in plain % (2011 +53 % / +41 %, 2016 +27 % / +42 %, 2019 -30 % / -27 %, 2020 +49 % / +25 %, 2021 -18 % / -26 %).</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Nitrogen does not follow the world price of the same year; it follows (weakly) the export price received for the previous crop (cash in hand), and state programmes: Bono Cafetalero 2020 = 25 188 t of fertiliser to 91 778 producers (USDA 2021), the year nitrogen use jumped 49 %.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Caution: part of the link can run the other way - growers fertilise more when flowering promises a big crop. For forecasting both readings point the same way: fertiliser bought Apr-Sep is a leading signal of the crop harvested from November. FAOSTAT stops in 2022: track fertiliser imports and urea prices instead.</t>
+          <t xml:space="preserve">Reading: nitrogen and output rise and fall together, in plain % (2011 +53 % / +41 %, 2016 +27 % / +42 %, 2019 -30 % / -27 %, 2020 +49 % / +25 %, 2021 -18 % / -26 %).</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Nitrogen does not follow the world price of the same year; it follows (weakly) the export price received for the previous crop (cash in hand), and state programmes: Bono Cafetalero 2020 = 25 188 t of fertiliser to 91 778 producers (USDA 2021), the year nitrogen use jumped 49 %.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Caution: part of the link can run the other way - growers fertilise more when flowering promises a big crop. For forecasting both readings point the same way: fertiliser bought Apr-Sep is a leading signal of the crop harvested from November. FAOSTAT stops in 2024 (2022 imputed): for 2025-26 track fertiliser imports and urea prices instead.</t>
         </is>
       </c>
     </row>
@@ -12004,7 +12058,7 @@
         <v>-0.14597005532086774</v>
       </c>
       <c r="E56" s="14">
-        <v>0.33813237352529496</v>
+        <v>0.35552889422115574</v>
       </c>
     </row>
     <row r="57">
@@ -12025,7 +12079,7 @@
         <v>-0.12102380613795989</v>
       </c>
       <c r="E57" s="14">
-        <v>0.47230553889222154</v>
+        <v>0.4549090181963607</v>
       </c>
     </row>
     <row r="58">
@@ -12046,7 +12100,7 @@
         <v>0.16206242211528962</v>
       </c>
       <c r="E58" s="14">
-        <v>0.28514297140571887</v>
+        <v>0.3027394521095781</v>
       </c>
     </row>
     <row r="59">
@@ -12067,7 +12121,7 @@
         <v>0.2652774445033983</v>
       </c>
       <c r="E59" s="14">
-        <v>0.10997800439912017</v>
+        <v>0.10137972405518897</v>
       </c>
     </row>
     <row r="60">
@@ -12088,7 +12142,7 @@
         <v>-0.295079173656936</v>
       </c>
       <c r="E60" s="14">
-        <v>0.052589482103579284</v>
+        <v>0.04839032193561288</v>
       </c>
     </row>
     <row r="61">
@@ -12109,7 +12163,7 @@
         <v>-0.13150030305448143</v>
       </c>
       <c r="E61" s="14">
-        <v>0.4277144571085783</v>
+        <v>0.4257148570285943</v>
       </c>
     </row>
     <row r="62">
@@ -12130,7 +12184,7 @@
         <v>-0.45284158573931876</v>
       </c>
       <c r="E62" s="14">
-        <v>0.002599480103979204</v>
+        <v>0.0015996800639872025</v>
       </c>
     </row>
     <row r="63">
@@ -12151,7 +12205,7 @@
         <v>-0.386901950622252</v>
       </c>
       <c r="E63" s="14">
-        <v>0.014997000599880024</v>
+        <v>0.015396920615876825</v>
       </c>
     </row>
     <row r="64">
@@ -12172,7 +12226,7 @@
         <v>-0.44034735086320853</v>
       </c>
       <c r="E64" s="14">
-        <v>0.0057988402319536095</v>
+        <v>0.008798240351929614</v>
       </c>
     </row>
     <row r="65">
@@ -12193,7 +12247,7 @@
         <v>-0.5281885471493315</v>
       </c>
       <c r="E65" s="14">
-        <v>0.0005998800239952009</v>
+        <v>0.0001999600079984003</v>
       </c>
     </row>
     <row r="66">
@@ -12214,7 +12268,7 @@
         <v>0.0457120796264875</v>
       </c>
       <c r="E66" s="14">
-        <v>0.7624475104979004</v>
+        <v>0.7676464707058588</v>
       </c>
     </row>
     <row r="67">

</xml_diff>